<commit_message>
Author: Гогунська Людмила; document image location in README
Co-authored-by: volodymyr-hohunskyi <volodymyr-hohunskyi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/shared/data/blog_import.xlsx
+++ b/shared/data/blog_import.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -747,7 +747,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -869,7 +869,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -991,7 +991,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Fun Dacha</t>
+          <t>Гогунська Людмила</t>
         </is>
       </c>
       <c r="G32" t="n">

</xml_diff>